<commit_message>
casee-v0.4.0-rc1: add native diagnostic runs
</commit_message>
<xml_diff>
--- a/docs/experiments/casee/results/casee_validation_summary.xlsx
+++ b/docs/experiments/casee/results/casee_validation_summary.xlsx
@@ -2938,9 +2938,15 @@
       <c r="G2" t="n">
         <v>0.18</v>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="H2" t="n">
+        <v>0.09546717</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-0.08453282999999999</v>
+      </c>
+      <c r="J2" t="n">
+        <v>8.453282999999999</v>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -2953,7 +2959,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -2983,9 +2989,15 @@
       <c r="G3" t="n">
         <v>0.59</v>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>0.20450579</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-0.3854942099999999</v>
+      </c>
+      <c r="J3" t="n">
+        <v>38.549421</v>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -2998,7 +3010,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3028,9 +3040,15 @@
       <c r="G4" t="n">
         <v>0.38</v>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>0.20486198</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-0.17513802</v>
+      </c>
+      <c r="J4" t="n">
+        <v>17.513802</v>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3043,7 +3061,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3073,9 +3091,15 @@
       <c r="G5" t="n">
         <v>0.32</v>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>0.06425537000000001</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.25574463</v>
+      </c>
+      <c r="J5" t="n">
+        <v>25.574463</v>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3088,7 +3112,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3118,9 +3142,15 @@
       <c r="G6" t="n">
         <v>0.3</v>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>0.08705723</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-0.21294277</v>
+      </c>
+      <c r="J6" t="n">
+        <v>21.294277</v>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3133,7 +3163,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3163,9 +3193,15 @@
       <c r="G7" t="n">
         <v>0.34</v>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>0.05495165</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-0.28504835</v>
+      </c>
+      <c r="J7" t="n">
+        <v>28.504835</v>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3178,7 +3214,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3208,9 +3244,15 @@
       <c r="G8" t="n">
         <v>0.26</v>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>0.13935074</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-0.12064926</v>
+      </c>
+      <c r="J8" t="n">
+        <v>12.064926</v>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3223,7 +3265,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3253,9 +3295,15 @@
       <c r="G9" t="n">
         <v>0.14</v>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>0.02378395</v>
+      </c>
+      <c r="I9" t="n">
+        <v>-0.11621605</v>
+      </c>
+      <c r="J9" t="n">
+        <v>11.621605</v>
+      </c>
       <c r="K9" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3268,7 +3316,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3298,9 +3346,15 @@
       <c r="G10" t="n">
         <v>0.12</v>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>0.13771719</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.01771718999999999</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1.771718999999999</v>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3313,7 +3367,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3343,9 +3397,15 @@
       <c r="G11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>0.16322637</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.06322637</v>
+      </c>
+      <c r="J11" t="n">
+        <v>6.322637</v>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3358,7 +3418,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3388,9 +3448,15 @@
       <c r="G12" t="n">
         <v>0.55</v>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>0.06055216</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-0.48944784</v>
+      </c>
+      <c r="J12" t="n">
+        <v>48.94478400000001</v>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3403,7 +3469,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3433,9 +3499,15 @@
       <c r="G13" t="n">
         <v>0.3</v>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>0.21425193</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-0.08574806999999998</v>
+      </c>
+      <c r="J13" t="n">
+        <v>8.574806999999998</v>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3448,7 +3520,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3478,9 +3550,15 @@
       <c r="G14" t="n">
         <v>0.59</v>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>0.20994979</v>
+      </c>
+      <c r="I14" t="n">
+        <v>-0.3800502099999999</v>
+      </c>
+      <c r="J14" t="n">
+        <v>38.00502099999999</v>
+      </c>
       <c r="K14" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3493,7 +3571,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3523,9 +3601,15 @@
       <c r="G15" t="n">
         <v>0.46</v>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>0.19744642</v>
+      </c>
+      <c r="I15" t="n">
+        <v>-0.26255358</v>
+      </c>
+      <c r="J15" t="n">
+        <v>26.255358</v>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3538,7 +3622,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3568,9 +3652,15 @@
       <c r="G16" t="n">
         <v>0.4</v>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>0.20340218</v>
+      </c>
+      <c r="I16" t="n">
+        <v>-0.19659782</v>
+      </c>
+      <c r="J16" t="n">
+        <v>19.659782</v>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3583,7 +3673,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3613,9 +3703,15 @@
       <c r="G17" t="n">
         <v>0.38</v>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>0.19801378</v>
+      </c>
+      <c r="I17" t="n">
+        <v>-0.18198622</v>
+      </c>
+      <c r="J17" t="n">
+        <v>18.198622</v>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3628,7 +3724,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3658,9 +3754,15 @@
       <c r="G18" t="n">
         <v>0.2</v>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>0.04666584</v>
+      </c>
+      <c r="I18" t="n">
+        <v>-0.15333416</v>
+      </c>
+      <c r="J18" t="n">
+        <v>15.333416</v>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3673,7 +3775,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3703,9 +3805,15 @@
       <c r="G19" t="n">
         <v>0.28</v>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>0.08527519</v>
+      </c>
+      <c r="I19" t="n">
+        <v>-0.19472481</v>
+      </c>
+      <c r="J19" t="n">
+        <v>19.472481</v>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3718,7 +3826,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3748,9 +3856,15 @@
       <c r="G20" t="n">
         <v>0.32</v>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>0.13612098</v>
+      </c>
+      <c r="I20" t="n">
+        <v>-0.18387902</v>
+      </c>
+      <c r="J20" t="n">
+        <v>18.387902</v>
+      </c>
       <c r="K20" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3763,7 +3877,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3793,9 +3907,15 @@
       <c r="G21" t="n">
         <v>0.2</v>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>0.10610108</v>
+      </c>
+      <c r="I21" t="n">
+        <v>-0.09389892000000001</v>
+      </c>
+      <c r="J21" t="n">
+        <v>9.389892000000001</v>
+      </c>
       <c r="K21" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3808,7 +3928,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3838,9 +3958,15 @@
       <c r="G22" t="n">
         <v>0.4</v>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>0.13523062</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-0.2647693800000001</v>
+      </c>
+      <c r="J22" t="n">
+        <v>26.476938</v>
+      </c>
       <c r="K22" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3853,7 +3979,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3883,9 +4009,15 @@
       <c r="G23" t="n">
         <v>0.59</v>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>0.07465586</v>
+      </c>
+      <c r="I23" t="n">
+        <v>-0.51534414</v>
+      </c>
+      <c r="J23" t="n">
+        <v>51.534414</v>
+      </c>
       <c r="K23" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3898,7 +4030,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3928,9 +4060,15 @@
       <c r="G24" t="n">
         <v>0.54</v>
       </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
+      <c r="H24" t="n">
+        <v>0.02505763</v>
+      </c>
+      <c r="I24" t="n">
+        <v>-0.51494237</v>
+      </c>
+      <c r="J24" t="n">
+        <v>51.494237</v>
+      </c>
       <c r="K24" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3943,7 +4081,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -3973,9 +4111,15 @@
       <c r="G25" t="n">
         <v>0.46</v>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
+      <c r="H25" t="n">
+        <v>0.19145018</v>
+      </c>
+      <c r="I25" t="n">
+        <v>-0.2685498200000001</v>
+      </c>
+      <c r="J25" t="n">
+        <v>26.85498200000001</v>
+      </c>
       <c r="K25" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -3988,7 +4132,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4018,9 +4162,15 @@
       <c r="G26" t="n">
         <v>0.52</v>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
+      <c r="H26" t="n">
+        <v>0.17377535</v>
+      </c>
+      <c r="I26" t="n">
+        <v>-0.34622465</v>
+      </c>
+      <c r="J26" t="n">
+        <v>34.62246500000001</v>
+      </c>
       <c r="K26" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4033,7 +4183,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4063,9 +4213,15 @@
       <c r="G27" t="n">
         <v>0.55</v>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>0.21925121</v>
+      </c>
+      <c r="I27" t="n">
+        <v>-0.33074879</v>
+      </c>
+      <c r="J27" t="n">
+        <v>33.074879</v>
+      </c>
       <c r="K27" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4078,7 +4234,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4108,9 +4264,15 @@
       <c r="G28" t="n">
         <v>0.48</v>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>0.1013118</v>
+      </c>
+      <c r="I28" t="n">
+        <v>-0.3786882</v>
+      </c>
+      <c r="J28" t="n">
+        <v>37.86882</v>
+      </c>
       <c r="K28" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4123,7 +4285,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4153,9 +4315,15 @@
       <c r="G29" t="n">
         <v>0.71</v>
       </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
+      <c r="H29" t="n">
+        <v>0.09312088</v>
+      </c>
+      <c r="I29" t="n">
+        <v>-0.61687912</v>
+      </c>
+      <c r="J29" t="n">
+        <v>61.687912</v>
+      </c>
       <c r="K29" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4168,7 +4336,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4198,9 +4366,15 @@
       <c r="G30" t="n">
         <v>0.61</v>
       </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
+      <c r="H30" t="n">
+        <v>0.24138681</v>
+      </c>
+      <c r="I30" t="n">
+        <v>-0.36861319</v>
+      </c>
+      <c r="J30" t="n">
+        <v>36.86131899999999</v>
+      </c>
       <c r="K30" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4213,7 +4387,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4243,9 +4417,15 @@
       <c r="G31" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
+      <c r="H31" t="n">
+        <v>0.11988474</v>
+      </c>
+      <c r="I31" t="n">
+        <v>-0.5701152599999999</v>
+      </c>
+      <c r="J31" t="n">
+        <v>57.01152599999999</v>
+      </c>
       <c r="K31" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4258,7 +4438,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4288,9 +4468,15 @@
       <c r="G32" t="n">
         <v>0.44</v>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
+      <c r="H32" t="n">
+        <v>0.08352166</v>
+      </c>
+      <c r="I32" t="n">
+        <v>-0.35647834</v>
+      </c>
+      <c r="J32" t="n">
+        <v>35.647834</v>
+      </c>
       <c r="K32" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4303,7 +4489,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4333,9 +4519,15 @@
       <c r="G33" t="n">
         <v>0.54</v>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
+      <c r="H33" t="n">
+        <v>0.01433129</v>
+      </c>
+      <c r="I33" t="n">
+        <v>-0.52566871</v>
+      </c>
+      <c r="J33" t="n">
+        <v>52.56687100000001</v>
+      </c>
       <c r="K33" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4348,7 +4540,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4378,9 +4570,15 @@
       <c r="G34" t="n">
         <v>0.52</v>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
+      <c r="H34" t="n">
+        <v>0.06945952</v>
+      </c>
+      <c r="I34" t="n">
+        <v>-0.45054048</v>
+      </c>
+      <c r="J34" t="n">
+        <v>45.054048</v>
+      </c>
       <c r="K34" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4393,7 +4591,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4423,9 +4621,15 @@
       <c r="G35" t="n">
         <v>0.32</v>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
+      <c r="H35" t="n">
+        <v>0.2129248</v>
+      </c>
+      <c r="I35" t="n">
+        <v>-0.1070752</v>
+      </c>
+      <c r="J35" t="n">
+        <v>10.70752</v>
+      </c>
       <c r="K35" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4438,7 +4642,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4468,9 +4672,15 @@
       <c r="G36" t="n">
         <v>0.5</v>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
+      <c r="H36" t="n">
+        <v>0.1905775</v>
+      </c>
+      <c r="I36" t="n">
+        <v>-0.3094225</v>
+      </c>
+      <c r="J36" t="n">
+        <v>30.94225</v>
+      </c>
       <c r="K36" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4483,7 +4693,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4513,9 +4723,15 @@
       <c r="G37" t="n">
         <v>0.32</v>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
+      <c r="H37" t="n">
+        <v>0.23709257</v>
+      </c>
+      <c r="I37" t="n">
+        <v>-0.08290743</v>
+      </c>
+      <c r="J37" t="n">
+        <v>8.290743000000001</v>
+      </c>
       <c r="K37" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4528,7 +4744,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4558,9 +4774,15 @@
       <c r="G38" t="n">
         <v>0.48</v>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
+      <c r="H38" t="n">
+        <v>0.20582877</v>
+      </c>
+      <c r="I38" t="n">
+        <v>-0.27417123</v>
+      </c>
+      <c r="J38" t="n">
+        <v>27.417123</v>
+      </c>
       <c r="K38" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4573,7 +4795,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4603,9 +4825,15 @@
       <c r="G39" t="n">
         <v>0.61</v>
       </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
+      <c r="H39" t="n">
+        <v>0.07605139</v>
+      </c>
+      <c r="I39" t="n">
+        <v>-0.5339486099999999</v>
+      </c>
+      <c r="J39" t="n">
+        <v>53.39486099999999</v>
+      </c>
       <c r="K39" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4618,7 +4846,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4648,9 +4876,15 @@
       <c r="G40" t="n">
         <v>0.26</v>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
+      <c r="H40" t="n">
+        <v>0.09354744</v>
+      </c>
+      <c r="I40" t="n">
+        <v>-0.16645256</v>
+      </c>
+      <c r="J40" t="n">
+        <v>16.645256</v>
+      </c>
       <c r="K40" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4663,7 +4897,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4693,9 +4927,15 @@
       <c r="G41" t="n">
         <v>0.38</v>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
+      <c r="H41" t="n">
+        <v>0.2135035</v>
+      </c>
+      <c r="I41" t="n">
+        <v>-0.1664965</v>
+      </c>
+      <c r="J41" t="n">
+        <v>16.64965</v>
+      </c>
       <c r="K41" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4708,7 +4948,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4738,9 +4978,15 @@
       <c r="G42" t="n">
         <v>0.46</v>
       </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
+      <c r="H42" t="n">
+        <v>0.20855558</v>
+      </c>
+      <c r="I42" t="n">
+        <v>-0.25144442</v>
+      </c>
+      <c r="J42" t="n">
+        <v>25.144442</v>
+      </c>
       <c r="K42" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4753,7 +4999,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4783,9 +5029,15 @@
       <c r="G43" t="n">
         <v>0.44</v>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
+      <c r="H43" t="n">
+        <v>0.08284068999999999</v>
+      </c>
+      <c r="I43" t="n">
+        <v>-0.35715931</v>
+      </c>
+      <c r="J43" t="n">
+        <v>35.715931</v>
+      </c>
       <c r="K43" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4798,7 +5050,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4828,9 +5080,15 @@
       <c r="G44" t="n">
         <v>0.3</v>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
+      <c r="H44" t="n">
+        <v>0.02021212</v>
+      </c>
+      <c r="I44" t="n">
+        <v>-0.27978788</v>
+      </c>
+      <c r="J44" t="n">
+        <v>27.978788</v>
+      </c>
       <c r="K44" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4843,7 +5101,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4873,9 +5131,15 @@
       <c r="G45" t="n">
         <v>0.46</v>
       </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
+      <c r="H45" t="n">
+        <v>0.01732341</v>
+      </c>
+      <c r="I45" t="n">
+        <v>-0.44267659</v>
+      </c>
+      <c r="J45" t="n">
+        <v>44.267659</v>
+      </c>
       <c r="K45" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4888,7 +5152,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4918,9 +5182,15 @@
       <c r="G46" t="n">
         <v>0.2</v>
       </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
+      <c r="H46" t="n">
+        <v>0.05640998</v>
+      </c>
+      <c r="I46" t="n">
+        <v>-0.14359002</v>
+      </c>
+      <c r="J46" t="n">
+        <v>14.359002</v>
+      </c>
       <c r="K46" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4933,7 +5203,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -4963,9 +5233,15 @@
       <c r="G47" t="n">
         <v>0.18</v>
       </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
+      <c r="H47" t="n">
+        <v>0.06605535</v>
+      </c>
+      <c r="I47" t="n">
+        <v>-0.11394465</v>
+      </c>
+      <c r="J47" t="n">
+        <v>11.394465</v>
+      </c>
       <c r="K47" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -4978,7 +5254,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5008,9 +5284,15 @@
       <c r="G48" t="n">
         <v>0.2</v>
       </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
+      <c r="H48" t="n">
+        <v>0.03055682</v>
+      </c>
+      <c r="I48" t="n">
+        <v>-0.16944318</v>
+      </c>
+      <c r="J48" t="n">
+        <v>16.944318</v>
+      </c>
       <c r="K48" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5023,7 +5305,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5053,9 +5335,15 @@
       <c r="G49" t="n">
         <v>0.36</v>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
+      <c r="H49" t="n">
+        <v>0.16870396</v>
+      </c>
+      <c r="I49" t="n">
+        <v>-0.19129604</v>
+      </c>
+      <c r="J49" t="n">
+        <v>19.129604</v>
+      </c>
       <c r="K49" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5068,7 +5356,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5098,9 +5386,15 @@
       <c r="G50" t="n">
         <v>0.3</v>
       </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
+      <c r="H50" t="n">
+        <v>0.09516602</v>
+      </c>
+      <c r="I50" t="n">
+        <v>-0.20483398</v>
+      </c>
+      <c r="J50" t="n">
+        <v>20.483398</v>
+      </c>
       <c r="K50" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5113,7 +5407,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5143,9 +5437,15 @@
       <c r="G51" t="n">
         <v>0.26</v>
       </c>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
+      <c r="H51" t="n">
+        <v>0.00465641</v>
+      </c>
+      <c r="I51" t="n">
+        <v>-0.25534359</v>
+      </c>
+      <c r="J51" t="n">
+        <v>25.534359</v>
+      </c>
       <c r="K51" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5158,7 +5458,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5188,9 +5488,15 @@
       <c r="G52" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
+      <c r="H52" t="n">
+        <v>0.13609306</v>
+      </c>
+      <c r="I52" t="n">
+        <v>-0.55390694</v>
+      </c>
+      <c r="J52" t="n">
+        <v>55.390694</v>
+      </c>
       <c r="K52" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5203,7 +5509,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5233,9 +5539,15 @@
       <c r="G53" t="n">
         <v>0.63</v>
       </c>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
+      <c r="H53" t="n">
+        <v>0.01473114</v>
+      </c>
+      <c r="I53" t="n">
+        <v>-0.61526886</v>
+      </c>
+      <c r="J53" t="n">
+        <v>61.526886</v>
+      </c>
       <c r="K53" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5248,7 +5560,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5278,9 +5590,15 @@
       <c r="G54" t="n">
         <v>0.57</v>
       </c>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
+      <c r="H54" t="n">
+        <v>0.05653114</v>
+      </c>
+      <c r="I54" t="n">
+        <v>-0.5134688599999999</v>
+      </c>
+      <c r="J54" t="n">
+        <v>51.34688599999999</v>
+      </c>
       <c r="K54" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5293,7 +5611,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5323,9 +5641,15 @@
       <c r="G55" t="n">
         <v>0.59</v>
       </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
+      <c r="H55" t="n">
+        <v>0.00708911</v>
+      </c>
+      <c r="I55" t="n">
+        <v>-0.58291089</v>
+      </c>
+      <c r="J55" t="n">
+        <v>58.291089</v>
+      </c>
       <c r="K55" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5338,7 +5662,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5368,9 +5692,15 @@
       <c r="G56" t="n">
         <v>0.38</v>
       </c>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
+      <c r="H56" t="n">
+        <v>0.12729215</v>
+      </c>
+      <c r="I56" t="n">
+        <v>-0.25270785</v>
+      </c>
+      <c r="J56" t="n">
+        <v>25.270785</v>
+      </c>
       <c r="K56" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5383,7 +5713,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5413,9 +5743,15 @@
       <c r="G57" t="n">
         <v>0.67</v>
       </c>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
+      <c r="H57" t="n">
+        <v>0.16200325</v>
+      </c>
+      <c r="I57" t="n">
+        <v>-0.50799675</v>
+      </c>
+      <c r="J57" t="n">
+        <v>50.799675</v>
+      </c>
       <c r="K57" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5428,7 +5764,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5458,9 +5794,15 @@
       <c r="G58" t="n">
         <v>0.34</v>
       </c>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
+      <c r="H58" t="n">
+        <v>0.16225573</v>
+      </c>
+      <c r="I58" t="n">
+        <v>-0.17774427</v>
+      </c>
+      <c r="J58" t="n">
+        <v>17.774427</v>
+      </c>
       <c r="K58" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5473,7 +5815,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5503,9 +5845,15 @@
       <c r="G59" t="n">
         <v>0.85</v>
       </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
+      <c r="H59" t="n">
+        <v>0.01434085</v>
+      </c>
+      <c r="I59" t="n">
+        <v>-0.83565915</v>
+      </c>
+      <c r="J59" t="n">
+        <v>83.565915</v>
+      </c>
       <c r="K59" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5518,7 +5866,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5548,9 +5896,15 @@
       <c r="G60" t="n">
         <v>0.42</v>
       </c>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
+      <c r="H60" t="n">
+        <v>0.11006569</v>
+      </c>
+      <c r="I60" t="n">
+        <v>-0.30993431</v>
+      </c>
+      <c r="J60" t="n">
+        <v>30.993431</v>
+      </c>
       <c r="K60" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5563,7 +5917,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5593,9 +5947,15 @@
       <c r="G61" t="n">
         <v>0.73</v>
       </c>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
+      <c r="H61" t="n">
+        <v>0.08737592</v>
+      </c>
+      <c r="I61" t="n">
+        <v>-0.64262408</v>
+      </c>
+      <c r="J61" t="n">
+        <v>64.26240800000001</v>
+      </c>
       <c r="K61" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5608,7 +5968,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5638,9 +5998,15 @@
       <c r="G62" t="n">
         <v>0.54</v>
       </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
+      <c r="H62" t="n">
+        <v>0.01822996</v>
+      </c>
+      <c r="I62" t="n">
+        <v>-0.52177004</v>
+      </c>
+      <c r="J62" t="n">
+        <v>52.177004</v>
+      </c>
       <c r="K62" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5653,7 +6019,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5683,9 +6049,15 @@
       <c r="G63" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
+      <c r="H63" t="n">
+        <v>0.02664088</v>
+      </c>
+      <c r="I63" t="n">
+        <v>-0.66335912</v>
+      </c>
+      <c r="J63" t="n">
+        <v>66.33591199999999</v>
+      </c>
       <c r="K63" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5698,7 +6070,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5728,9 +6100,15 @@
       <c r="G64" t="n">
         <v>0.4</v>
       </c>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
+      <c r="H64" t="n">
+        <v>0.0952384</v>
+      </c>
+      <c r="I64" t="n">
+        <v>-0.3047616</v>
+      </c>
+      <c r="J64" t="n">
+        <v>30.47616</v>
+      </c>
       <c r="K64" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5743,7 +6121,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5773,9 +6151,15 @@
       <c r="G65" t="n">
         <v>0.44</v>
       </c>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
+      <c r="H65" t="n">
+        <v>0.19786003</v>
+      </c>
+      <c r="I65" t="n">
+        <v>-0.24213997</v>
+      </c>
+      <c r="J65" t="n">
+        <v>24.213997</v>
+      </c>
       <c r="K65" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5788,7 +6172,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5818,9 +6202,15 @@
       <c r="G66" t="n">
         <v>0.3</v>
       </c>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
+      <c r="H66" t="n">
+        <v>0.09074802</v>
+      </c>
+      <c r="I66" t="n">
+        <v>-0.20925198</v>
+      </c>
+      <c r="J66" t="n">
+        <v>20.925198</v>
+      </c>
       <c r="K66" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5833,7 +6223,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5863,9 +6253,15 @@
       <c r="G67" t="n">
         <v>0.32</v>
       </c>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
+      <c r="H67" t="n">
+        <v>0.07100185000000001</v>
+      </c>
+      <c r="I67" t="n">
+        <v>-0.24899815</v>
+      </c>
+      <c r="J67" t="n">
+        <v>24.899815</v>
+      </c>
       <c r="K67" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5878,7 +6274,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5908,9 +6304,15 @@
       <c r="G68" t="n">
         <v>0.5</v>
       </c>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
+      <c r="H68" t="n">
+        <v>0.19550085</v>
+      </c>
+      <c r="I68" t="n">
+        <v>-0.30449915</v>
+      </c>
+      <c r="J68" t="n">
+        <v>30.449915</v>
+      </c>
       <c r="K68" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5923,7 +6325,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5953,9 +6355,15 @@
       <c r="G69" t="n">
         <v>0.28</v>
       </c>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
+      <c r="H69" t="n">
+        <v>0.06899553999999999</v>
+      </c>
+      <c r="I69" t="n">
+        <v>-0.21100446</v>
+      </c>
+      <c r="J69" t="n">
+        <v>21.100446</v>
+      </c>
       <c r="K69" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -5968,7 +6376,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -5998,9 +6406,15 @@
       <c r="G70" t="n">
         <v>0.24</v>
       </c>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
+      <c r="H70" t="n">
+        <v>0.11074632</v>
+      </c>
+      <c r="I70" t="n">
+        <v>-0.12925368</v>
+      </c>
+      <c r="J70" t="n">
+        <v>12.925368</v>
+      </c>
       <c r="K70" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -6013,7 +6427,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -6043,9 +6457,15 @@
       <c r="G71" t="n">
         <v>0.34</v>
       </c>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
+      <c r="H71" t="n">
+        <v>0.02156874</v>
+      </c>
+      <c r="I71" t="n">
+        <v>-0.31843126</v>
+      </c>
+      <c r="J71" t="n">
+        <v>31.84312600000001</v>
+      </c>
       <c r="K71" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -6058,7 +6478,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -6088,9 +6508,15 @@
       <c r="G72" t="n">
         <v>0.5</v>
       </c>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
+      <c r="H72" t="n">
+        <v>0.21179647</v>
+      </c>
+      <c r="I72" t="n">
+        <v>-0.28820353</v>
+      </c>
+      <c r="J72" t="n">
+        <v>28.820353</v>
+      </c>
       <c r="K72" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -6103,7 +6529,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -6133,9 +6559,15 @@
       <c r="G73" t="n">
         <v>0.38</v>
       </c>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
+      <c r="H73" t="n">
+        <v>0.01815125</v>
+      </c>
+      <c r="I73" t="n">
+        <v>-0.36184875</v>
+      </c>
+      <c r="J73" t="n">
+        <v>36.184875</v>
+      </c>
       <c r="K73" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -6148,7 +6580,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -6178,9 +6610,15 @@
       <c r="G74" t="n">
         <v>0.52</v>
       </c>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
+      <c r="H74" t="n">
+        <v>0.11149217</v>
+      </c>
+      <c r="I74" t="n">
+        <v>-0.40850783</v>
+      </c>
+      <c r="J74" t="n">
+        <v>40.850783</v>
+      </c>
       <c r="K74" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -6193,7 +6631,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -6223,9 +6661,15 @@
       <c r="G75" t="n">
         <v>0.26</v>
       </c>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
+      <c r="H75" t="n">
+        <v>0.01979482</v>
+      </c>
+      <c r="I75" t="n">
+        <v>-0.24020518</v>
+      </c>
+      <c r="J75" t="n">
+        <v>24.020518</v>
+      </c>
       <c r="K75" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -6238,7 +6682,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -6268,9 +6712,15 @@
       <c r="G76" t="n">
         <v>0.63</v>
       </c>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
+      <c r="H76" t="n">
+        <v>0.01504631</v>
+      </c>
+      <c r="I76" t="n">
+        <v>-0.61495369</v>
+      </c>
+      <c r="J76" t="n">
+        <v>61.495369</v>
+      </c>
       <c r="K76" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -6283,7 +6733,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -6313,9 +6763,15 @@
       <c r="G77" t="n">
         <v>0.5</v>
       </c>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
+      <c r="H77" t="n">
+        <v>0.00939399</v>
+      </c>
+      <c r="I77" t="n">
+        <v>-0.49060601</v>
+      </c>
+      <c r="J77" t="n">
+        <v>49.060601</v>
+      </c>
       <c r="K77" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -6328,7 +6784,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -6358,9 +6814,15 @@
       <c r="G78" t="n">
         <v>0.46</v>
       </c>
-      <c r="H78" t="inlineStr"/>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
+      <c r="H78" t="n">
+        <v>0.11601727</v>
+      </c>
+      <c r="I78" t="n">
+        <v>-0.34398273</v>
+      </c>
+      <c r="J78" t="n">
+        <v>34.398273</v>
+      </c>
       <c r="K78" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -6373,7 +6835,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -6403,9 +6865,15 @@
       <c r="G79" t="n">
         <v>0.28</v>
       </c>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
+      <c r="H79" t="n">
+        <v>0.13797679</v>
+      </c>
+      <c r="I79" t="n">
+        <v>-0.14202321</v>
+      </c>
+      <c r="J79" t="n">
+        <v>14.202321</v>
+      </c>
       <c r="K79" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -6418,7 +6886,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -6448,9 +6916,15 @@
       <c r="G80" t="n">
         <v>0.32</v>
       </c>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
+      <c r="H80" t="n">
+        <v>0.1470067</v>
+      </c>
+      <c r="I80" t="n">
+        <v>-0.1729933</v>
+      </c>
+      <c r="J80" t="n">
+        <v>17.29933</v>
+      </c>
       <c r="K80" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -6463,7 +6937,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>
@@ -6493,9 +6967,15 @@
       <c r="G81" t="n">
         <v>0.54</v>
       </c>
-      <c r="H81" t="inlineStr"/>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
+      <c r="H81" t="n">
+        <v>0.09691590999999999</v>
+      </c>
+      <c r="I81" t="n">
+        <v>-0.44308409</v>
+      </c>
+      <c r="J81" t="n">
+        <v>44.308409</v>
+      </c>
       <c r="K81" t="inlineStr">
         <is>
           <t>raw_trilinear</t>
@@ -6508,7 +6988,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>newly_run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
casee-v0.4.0-rc1: add nu diagnostics
</commit_message>
<xml_diff>
--- a/docs/experiments/casee/results/casee_validation_summary.xlsx
+++ b/docs/experiments/casee/results/casee_validation_summary.xlsx
@@ -2939,13 +2939,13 @@
         <v>0.18</v>
       </c>
       <c r="H2" t="n">
-        <v>0.09546717</v>
+        <v>0.20830754</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.08453282999999999</v>
+        <v>0.02830754000000002</v>
       </c>
       <c r="J2" t="n">
-        <v>8.453282999999999</v>
+        <v>2.830754000000002</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -2990,13 +2990,13 @@
         <v>0.59</v>
       </c>
       <c r="H3" t="n">
-        <v>0.20450579</v>
+        <v>0.32874972</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.3854942099999999</v>
+        <v>-0.2612502799999999</v>
       </c>
       <c r="J3" t="n">
-        <v>38.549421</v>
+        <v>26.12502799999999</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -3041,13 +3041,13 @@
         <v>0.38</v>
       </c>
       <c r="H4" t="n">
-        <v>0.20486198</v>
+        <v>0.27719049</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.17513802</v>
+        <v>-0.10280951</v>
       </c>
       <c r="J4" t="n">
-        <v>17.513802</v>
+        <v>10.280951</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -3092,13 +3092,13 @@
         <v>0.32</v>
       </c>
       <c r="H5" t="n">
-        <v>0.06425537000000001</v>
+        <v>0.03532374</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.25574463</v>
+        <v>-0.28467626</v>
       </c>
       <c r="J5" t="n">
-        <v>25.574463</v>
+        <v>28.467626</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -3143,13 +3143,13 @@
         <v>0.3</v>
       </c>
       <c r="H6" t="n">
-        <v>0.08705723</v>
+        <v>0.16671328</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.21294277</v>
+        <v>-0.13328672</v>
       </c>
       <c r="J6" t="n">
-        <v>21.294277</v>
+        <v>13.328672</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -3194,13 +3194,13 @@
         <v>0.34</v>
       </c>
       <c r="H7" t="n">
-        <v>0.05495165</v>
+        <v>0.11874212</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.28504835</v>
+        <v>-0.22125788</v>
       </c>
       <c r="J7" t="n">
-        <v>28.504835</v>
+        <v>22.125788</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -3245,13 +3245,13 @@
         <v>0.26</v>
       </c>
       <c r="H8" t="n">
-        <v>0.13935074</v>
+        <v>0.25316522</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.12064926</v>
+        <v>-0.006834779999999985</v>
       </c>
       <c r="J8" t="n">
-        <v>12.064926</v>
+        <v>0.6834779999999985</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         <v>0.14</v>
       </c>
       <c r="H9" t="n">
-        <v>0.02378395</v>
+        <v>0.04925373</v>
       </c>
       <c r="I9" t="n">
-        <v>-0.11621605</v>
+        <v>-0.09074627000000002</v>
       </c>
       <c r="J9" t="n">
-        <v>11.621605</v>
+        <v>9.074627000000001</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -3347,13 +3347,13 @@
         <v>0.12</v>
       </c>
       <c r="H10" t="n">
-        <v>0.13771719</v>
+        <v>0.08338690999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>0.01771718999999999</v>
+        <v>-0.03661309</v>
       </c>
       <c r="J10" t="n">
-        <v>1.771718999999999</v>
+        <v>3.661309</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -3398,13 +3398,13 @@
         <v>0.1</v>
       </c>
       <c r="H11" t="n">
-        <v>0.16322637</v>
+        <v>0.31200519</v>
       </c>
       <c r="I11" t="n">
-        <v>0.06322637</v>
+        <v>0.21200519</v>
       </c>
       <c r="J11" t="n">
-        <v>6.322637</v>
+        <v>21.200519</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -3449,13 +3449,13 @@
         <v>0.55</v>
       </c>
       <c r="H12" t="n">
-        <v>0.06055216</v>
+        <v>0.22062139</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.48944784</v>
+        <v>-0.32937861</v>
       </c>
       <c r="J12" t="n">
-        <v>48.94478400000001</v>
+        <v>32.937861</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -3500,13 +3500,13 @@
         <v>0.3</v>
       </c>
       <c r="H13" t="n">
-        <v>0.21425193</v>
+        <v>0.2657773</v>
       </c>
       <c r="I13" t="n">
-        <v>-0.08574806999999998</v>
+        <v>-0.03422269999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>8.574806999999998</v>
+        <v>3.422269999999999</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -3551,13 +3551,13 @@
         <v>0.59</v>
       </c>
       <c r="H14" t="n">
-        <v>0.20994979</v>
+        <v>0.11199946</v>
       </c>
       <c r="I14" t="n">
-        <v>-0.3800502099999999</v>
+        <v>-0.47800054</v>
       </c>
       <c r="J14" t="n">
-        <v>38.00502099999999</v>
+        <v>47.800054</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -3602,13 +3602,13 @@
         <v>0.46</v>
       </c>
       <c r="H15" t="n">
-        <v>0.19744642</v>
+        <v>0.37454433</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.26255358</v>
+        <v>-0.08545567000000004</v>
       </c>
       <c r="J15" t="n">
-        <v>26.255358</v>
+        <v>8.545567000000004</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -3653,13 +3653,13 @@
         <v>0.4</v>
       </c>
       <c r="H16" t="n">
-        <v>0.20340218</v>
+        <v>0.384069</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.19659782</v>
+        <v>-0.01593100000000003</v>
       </c>
       <c r="J16" t="n">
-        <v>19.659782</v>
+        <v>1.593100000000003</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -3704,13 +3704,13 @@
         <v>0.38</v>
       </c>
       <c r="H17" t="n">
-        <v>0.19801378</v>
+        <v>0.23438932</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.18198622</v>
+        <v>-0.14561068</v>
       </c>
       <c r="J17" t="n">
-        <v>18.198622</v>
+        <v>14.561068</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -3755,13 +3755,13 @@
         <v>0.2</v>
       </c>
       <c r="H18" t="n">
-        <v>0.04666584</v>
+        <v>0.09064137</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.15333416</v>
+        <v>-0.10935863</v>
       </c>
       <c r="J18" t="n">
-        <v>15.333416</v>
+        <v>10.935863</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -3806,13 +3806,13 @@
         <v>0.28</v>
       </c>
       <c r="H19" t="n">
-        <v>0.08527519</v>
+        <v>0.16247229</v>
       </c>
       <c r="I19" t="n">
-        <v>-0.19472481</v>
+        <v>-0.11752771</v>
       </c>
       <c r="J19" t="n">
-        <v>19.472481</v>
+        <v>11.752771</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -3857,13 +3857,13 @@
         <v>0.32</v>
       </c>
       <c r="H20" t="n">
-        <v>0.13612098</v>
+        <v>0.03496582</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.18387902</v>
+        <v>-0.28503418</v>
       </c>
       <c r="J20" t="n">
-        <v>18.387902</v>
+        <v>28.503418</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -3908,13 +3908,13 @@
         <v>0.2</v>
       </c>
       <c r="H21" t="n">
-        <v>0.10610108</v>
+        <v>0.18146655</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.09389892000000001</v>
+        <v>-0.01853345000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>9.389892000000001</v>
+        <v>1.853345000000001</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -3959,13 +3959,13 @@
         <v>0.4</v>
       </c>
       <c r="H22" t="n">
-        <v>0.13523062</v>
+        <v>0.2651739</v>
       </c>
       <c r="I22" t="n">
-        <v>-0.2647693800000001</v>
+        <v>-0.1348261</v>
       </c>
       <c r="J22" t="n">
-        <v>26.476938</v>
+        <v>13.48261</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -4010,13 +4010,13 @@
         <v>0.59</v>
       </c>
       <c r="H23" t="n">
-        <v>0.07465586</v>
+        <v>0.16242976</v>
       </c>
       <c r="I23" t="n">
-        <v>-0.51534414</v>
+        <v>-0.42757024</v>
       </c>
       <c r="J23" t="n">
-        <v>51.534414</v>
+        <v>42.757024</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -4061,13 +4061,13 @@
         <v>0.54</v>
       </c>
       <c r="H24" t="n">
-        <v>0.02505763</v>
+        <v>0.15774745</v>
       </c>
       <c r="I24" t="n">
-        <v>-0.51494237</v>
+        <v>-0.38225255</v>
       </c>
       <c r="J24" t="n">
-        <v>51.494237</v>
+        <v>38.225255</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -4112,13 +4112,13 @@
         <v>0.46</v>
       </c>
       <c r="H25" t="n">
-        <v>0.19145018</v>
+        <v>0.19116407</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.2685498200000001</v>
+        <v>-0.2688359300000001</v>
       </c>
       <c r="J25" t="n">
-        <v>26.85498200000001</v>
+        <v>26.883593</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -4163,13 +4163,13 @@
         <v>0.52</v>
       </c>
       <c r="H26" t="n">
-        <v>0.17377535</v>
+        <v>0.38581118</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.34622465</v>
+        <v>-0.13418882</v>
       </c>
       <c r="J26" t="n">
-        <v>34.62246500000001</v>
+        <v>13.418882</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -4214,13 +4214,13 @@
         <v>0.55</v>
       </c>
       <c r="H27" t="n">
-        <v>0.21925121</v>
+        <v>0.35554295</v>
       </c>
       <c r="I27" t="n">
-        <v>-0.33074879</v>
+        <v>-0.19445705</v>
       </c>
       <c r="J27" t="n">
-        <v>33.074879</v>
+        <v>19.445705</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -4265,13 +4265,13 @@
         <v>0.48</v>
       </c>
       <c r="H28" t="n">
-        <v>0.1013118</v>
+        <v>0.19027389</v>
       </c>
       <c r="I28" t="n">
-        <v>-0.3786882</v>
+        <v>-0.28972611</v>
       </c>
       <c r="J28" t="n">
-        <v>37.86882</v>
+        <v>28.972611</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -4316,13 +4316,13 @@
         <v>0.71</v>
       </c>
       <c r="H29" t="n">
-        <v>0.09312088</v>
+        <v>0.39362757</v>
       </c>
       <c r="I29" t="n">
-        <v>-0.61687912</v>
+        <v>-0.31637243</v>
       </c>
       <c r="J29" t="n">
-        <v>61.687912</v>
+        <v>31.637243</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -4367,13 +4367,13 @@
         <v>0.61</v>
       </c>
       <c r="H30" t="n">
-        <v>0.24138681</v>
+        <v>0.54752525</v>
       </c>
       <c r="I30" t="n">
-        <v>-0.36861319</v>
+        <v>-0.06247475000000002</v>
       </c>
       <c r="J30" t="n">
-        <v>36.86131899999999</v>
+        <v>6.247475000000002</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -4418,13 +4418,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="H31" t="n">
-        <v>0.11988474</v>
+        <v>0.18938433</v>
       </c>
       <c r="I31" t="n">
-        <v>-0.5701152599999999</v>
+        <v>-0.50061567</v>
       </c>
       <c r="J31" t="n">
-        <v>57.01152599999999</v>
+        <v>50.061567</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -4469,13 +4469,13 @@
         <v>0.44</v>
       </c>
       <c r="H32" t="n">
-        <v>0.08352166</v>
+        <v>0.09889763999999999</v>
       </c>
       <c r="I32" t="n">
-        <v>-0.35647834</v>
+        <v>-0.34110236</v>
       </c>
       <c r="J32" t="n">
-        <v>35.647834</v>
+        <v>34.110236</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -4520,13 +4520,13 @@
         <v>0.54</v>
       </c>
       <c r="H33" t="n">
-        <v>0.01433129</v>
+        <v>0.20961041</v>
       </c>
       <c r="I33" t="n">
-        <v>-0.52566871</v>
+        <v>-0.33038959</v>
       </c>
       <c r="J33" t="n">
-        <v>52.56687100000001</v>
+        <v>33.038959</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -4571,13 +4571,13 @@
         <v>0.52</v>
       </c>
       <c r="H34" t="n">
-        <v>0.06945952</v>
+        <v>0.52939261</v>
       </c>
       <c r="I34" t="n">
-        <v>-0.45054048</v>
+        <v>0.009392610000000023</v>
       </c>
       <c r="J34" t="n">
-        <v>45.054048</v>
+        <v>0.9392610000000023</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -4622,13 +4622,13 @@
         <v>0.32</v>
       </c>
       <c r="H35" t="n">
-        <v>0.2129248</v>
+        <v>0.43110631</v>
       </c>
       <c r="I35" t="n">
-        <v>-0.1070752</v>
+        <v>0.11110631</v>
       </c>
       <c r="J35" t="n">
-        <v>10.70752</v>
+        <v>11.110631</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
@@ -4673,13 +4673,13 @@
         <v>0.5</v>
       </c>
       <c r="H36" t="n">
-        <v>0.1905775</v>
+        <v>0.39907543</v>
       </c>
       <c r="I36" t="n">
-        <v>-0.3094225</v>
+        <v>-0.10092457</v>
       </c>
       <c r="J36" t="n">
-        <v>30.94225</v>
+        <v>10.092457</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -4724,13 +4724,13 @@
         <v>0.32</v>
       </c>
       <c r="H37" t="n">
-        <v>0.23709257</v>
+        <v>0.42693671</v>
       </c>
       <c r="I37" t="n">
-        <v>-0.08290743</v>
+        <v>0.10693671</v>
       </c>
       <c r="J37" t="n">
-        <v>8.290743000000001</v>
+        <v>10.693671</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -4775,13 +4775,13 @@
         <v>0.48</v>
       </c>
       <c r="H38" t="n">
-        <v>0.20582877</v>
+        <v>0.31255821</v>
       </c>
       <c r="I38" t="n">
-        <v>-0.27417123</v>
+        <v>-0.16744179</v>
       </c>
       <c r="J38" t="n">
-        <v>27.417123</v>
+        <v>16.744179</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -4826,13 +4826,13 @@
         <v>0.61</v>
       </c>
       <c r="H39" t="n">
-        <v>0.07605139</v>
+        <v>0.11995387</v>
       </c>
       <c r="I39" t="n">
-        <v>-0.5339486099999999</v>
+        <v>-0.49004613</v>
       </c>
       <c r="J39" t="n">
-        <v>53.39486099999999</v>
+        <v>49.004613</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -4877,13 +4877,13 @@
         <v>0.26</v>
       </c>
       <c r="H40" t="n">
-        <v>0.09354744</v>
+        <v>0.36592446</v>
       </c>
       <c r="I40" t="n">
-        <v>-0.16645256</v>
+        <v>0.10592446</v>
       </c>
       <c r="J40" t="n">
-        <v>16.645256</v>
+        <v>10.592446</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -4928,13 +4928,13 @@
         <v>0.38</v>
       </c>
       <c r="H41" t="n">
-        <v>0.2135035</v>
+        <v>0.07938853</v>
       </c>
       <c r="I41" t="n">
-        <v>-0.1664965</v>
+        <v>-0.30061147</v>
       </c>
       <c r="J41" t="n">
-        <v>16.64965</v>
+        <v>30.061147</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -4979,13 +4979,13 @@
         <v>0.46</v>
       </c>
       <c r="H42" t="n">
-        <v>0.20855558</v>
+        <v>0.10755455</v>
       </c>
       <c r="I42" t="n">
-        <v>-0.25144442</v>
+        <v>-0.35244545</v>
       </c>
       <c r="J42" t="n">
-        <v>25.144442</v>
+        <v>35.244545</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -5030,13 +5030,13 @@
         <v>0.44</v>
       </c>
       <c r="H43" t="n">
-        <v>0.08284068999999999</v>
+        <v>0.11130642</v>
       </c>
       <c r="I43" t="n">
-        <v>-0.35715931</v>
+        <v>-0.32869358</v>
       </c>
       <c r="J43" t="n">
-        <v>35.715931</v>
+        <v>32.869358</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -5081,13 +5081,13 @@
         <v>0.3</v>
       </c>
       <c r="H44" t="n">
-        <v>0.02021212</v>
+        <v>0.1573176</v>
       </c>
       <c r="I44" t="n">
-        <v>-0.27978788</v>
+        <v>-0.1426824</v>
       </c>
       <c r="J44" t="n">
-        <v>27.978788</v>
+        <v>14.26824</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -5132,13 +5132,13 @@
         <v>0.46</v>
       </c>
       <c r="H45" t="n">
-        <v>0.01732341</v>
+        <v>0.21231887</v>
       </c>
       <c r="I45" t="n">
-        <v>-0.44267659</v>
+        <v>-0.24768113</v>
       </c>
       <c r="J45" t="n">
-        <v>44.267659</v>
+        <v>24.768113</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -5183,13 +5183,13 @@
         <v>0.2</v>
       </c>
       <c r="H46" t="n">
-        <v>0.05640998</v>
+        <v>0.27860525</v>
       </c>
       <c r="I46" t="n">
-        <v>-0.14359002</v>
+        <v>0.07860525000000002</v>
       </c>
       <c r="J46" t="n">
-        <v>14.359002</v>
+        <v>7.860525000000002</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
@@ -5234,13 +5234,13 @@
         <v>0.18</v>
       </c>
       <c r="H47" t="n">
-        <v>0.06605535</v>
+        <v>0.35965863</v>
       </c>
       <c r="I47" t="n">
-        <v>-0.11394465</v>
+        <v>0.17965863</v>
       </c>
       <c r="J47" t="n">
-        <v>11.394465</v>
+        <v>17.965863</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
@@ -5285,13 +5285,13 @@
         <v>0.2</v>
       </c>
       <c r="H48" t="n">
-        <v>0.03055682</v>
+        <v>0.00147794</v>
       </c>
       <c r="I48" t="n">
-        <v>-0.16944318</v>
+        <v>-0.19852206</v>
       </c>
       <c r="J48" t="n">
-        <v>16.944318</v>
+        <v>19.852206</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -5336,13 +5336,13 @@
         <v>0.36</v>
       </c>
       <c r="H49" t="n">
-        <v>0.16870396</v>
+        <v>0.336626</v>
       </c>
       <c r="I49" t="n">
-        <v>-0.19129604</v>
+        <v>-0.02337400000000001</v>
       </c>
       <c r="J49" t="n">
-        <v>19.129604</v>
+        <v>2.337400000000001</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
@@ -5387,13 +5387,13 @@
         <v>0.3</v>
       </c>
       <c r="H50" t="n">
-        <v>0.09516602</v>
+        <v>0.26429585</v>
       </c>
       <c r="I50" t="n">
-        <v>-0.20483398</v>
+        <v>-0.03570414999999999</v>
       </c>
       <c r="J50" t="n">
-        <v>20.483398</v>
+        <v>3.570414999999999</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
@@ -5438,13 +5438,13 @@
         <v>0.26</v>
       </c>
       <c r="H51" t="n">
-        <v>0.00465641</v>
+        <v>0.02155509</v>
       </c>
       <c r="I51" t="n">
-        <v>-0.25534359</v>
+        <v>-0.23844491</v>
       </c>
       <c r="J51" t="n">
-        <v>25.534359</v>
+        <v>23.844491</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -5489,13 +5489,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="H52" t="n">
-        <v>0.13609306</v>
+        <v>0.26060797</v>
       </c>
       <c r="I52" t="n">
-        <v>-0.55390694</v>
+        <v>-0.4293920299999999</v>
       </c>
       <c r="J52" t="n">
-        <v>55.390694</v>
+        <v>42.93920299999999</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -5540,13 +5540,13 @@
         <v>0.63</v>
       </c>
       <c r="H53" t="n">
-        <v>0.01473114</v>
+        <v>0.09783202000000001</v>
       </c>
       <c r="I53" t="n">
-        <v>-0.61526886</v>
+        <v>-0.53216798</v>
       </c>
       <c r="J53" t="n">
-        <v>61.526886</v>
+        <v>53.216798</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -5591,13 +5591,13 @@
         <v>0.57</v>
       </c>
       <c r="H54" t="n">
-        <v>0.05653114</v>
+        <v>0.16324099</v>
       </c>
       <c r="I54" t="n">
-        <v>-0.5134688599999999</v>
+        <v>-0.4067590099999999</v>
       </c>
       <c r="J54" t="n">
-        <v>51.34688599999999</v>
+        <v>40.67590099999999</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -5642,13 +5642,13 @@
         <v>0.59</v>
       </c>
       <c r="H55" t="n">
-        <v>0.00708911</v>
+        <v>0.04225041</v>
       </c>
       <c r="I55" t="n">
-        <v>-0.58291089</v>
+        <v>-0.54774959</v>
       </c>
       <c r="J55" t="n">
-        <v>58.291089</v>
+        <v>54.774959</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -5693,13 +5693,13 @@
         <v>0.38</v>
       </c>
       <c r="H56" t="n">
-        <v>0.12729215</v>
+        <v>0.29619185</v>
       </c>
       <c r="I56" t="n">
-        <v>-0.25270785</v>
+        <v>-0.08380815000000003</v>
       </c>
       <c r="J56" t="n">
-        <v>25.270785</v>
+        <v>8.380815000000002</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
@@ -5744,13 +5744,13 @@
         <v>0.67</v>
       </c>
       <c r="H57" t="n">
-        <v>0.16200325</v>
+        <v>0.20379514</v>
       </c>
       <c r="I57" t="n">
-        <v>-0.50799675</v>
+        <v>-0.4662048600000001</v>
       </c>
       <c r="J57" t="n">
-        <v>50.799675</v>
+        <v>46.62048600000001</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
@@ -5795,13 +5795,13 @@
         <v>0.34</v>
       </c>
       <c r="H58" t="n">
-        <v>0.16225573</v>
+        <v>0.38460754</v>
       </c>
       <c r="I58" t="n">
-        <v>-0.17774427</v>
+        <v>0.04460754</v>
       </c>
       <c r="J58" t="n">
-        <v>17.774427</v>
+        <v>4.460754</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -5846,13 +5846,13 @@
         <v>0.85</v>
       </c>
       <c r="H59" t="n">
-        <v>0.01434085</v>
+        <v>0.10843476</v>
       </c>
       <c r="I59" t="n">
-        <v>-0.83565915</v>
+        <v>-0.74156524</v>
       </c>
       <c r="J59" t="n">
-        <v>83.565915</v>
+        <v>74.156524</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
@@ -5897,13 +5897,13 @@
         <v>0.42</v>
       </c>
       <c r="H60" t="n">
-        <v>0.11006569</v>
+        <v>0.13367753</v>
       </c>
       <c r="I60" t="n">
-        <v>-0.30993431</v>
+        <v>-0.28632247</v>
       </c>
       <c r="J60" t="n">
-        <v>30.993431</v>
+        <v>28.632247</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
@@ -5948,13 +5948,13 @@
         <v>0.73</v>
       </c>
       <c r="H61" t="n">
-        <v>0.08737592</v>
+        <v>0.39983383</v>
       </c>
       <c r="I61" t="n">
-        <v>-0.64262408</v>
+        <v>-0.33016617</v>
       </c>
       <c r="J61" t="n">
-        <v>64.26240800000001</v>
+        <v>33.016617</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
@@ -5999,13 +5999,13 @@
         <v>0.54</v>
       </c>
       <c r="H62" t="n">
-        <v>0.01822996</v>
+        <v>0.01660191</v>
       </c>
       <c r="I62" t="n">
-        <v>-0.52177004</v>
+        <v>-0.52339809</v>
       </c>
       <c r="J62" t="n">
-        <v>52.177004</v>
+        <v>52.339809</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -6050,13 +6050,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="H63" t="n">
-        <v>0.02664088</v>
+        <v>0.02344557</v>
       </c>
       <c r="I63" t="n">
-        <v>-0.66335912</v>
+        <v>-0.6665544299999999</v>
       </c>
       <c r="J63" t="n">
-        <v>66.33591199999999</v>
+        <v>66.65544299999999</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -6101,13 +6101,13 @@
         <v>0.4</v>
       </c>
       <c r="H64" t="n">
-        <v>0.0952384</v>
+        <v>0.25829743</v>
       </c>
       <c r="I64" t="n">
-        <v>-0.3047616</v>
+        <v>-0.14170257</v>
       </c>
       <c r="J64" t="n">
-        <v>30.47616</v>
+        <v>14.170257</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
@@ -6152,13 +6152,13 @@
         <v>0.44</v>
       </c>
       <c r="H65" t="n">
-        <v>0.19786003</v>
+        <v>0.33534344</v>
       </c>
       <c r="I65" t="n">
-        <v>-0.24213997</v>
+        <v>-0.10465656</v>
       </c>
       <c r="J65" t="n">
-        <v>24.213997</v>
+        <v>10.465656</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -6203,13 +6203,13 @@
         <v>0.3</v>
       </c>
       <c r="H66" t="n">
-        <v>0.09074802</v>
+        <v>0.05556118</v>
       </c>
       <c r="I66" t="n">
-        <v>-0.20925198</v>
+        <v>-0.24443882</v>
       </c>
       <c r="J66" t="n">
-        <v>20.925198</v>
+        <v>24.443882</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
@@ -6254,13 +6254,13 @@
         <v>0.32</v>
       </c>
       <c r="H67" t="n">
-        <v>0.07100185000000001</v>
+        <v>0.01333601</v>
       </c>
       <c r="I67" t="n">
-        <v>-0.24899815</v>
+        <v>-0.30666399</v>
       </c>
       <c r="J67" t="n">
-        <v>24.899815</v>
+        <v>30.666399</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -6305,13 +6305,13 @@
         <v>0.5</v>
       </c>
       <c r="H68" t="n">
-        <v>0.19550085</v>
+        <v>0.46313159</v>
       </c>
       <c r="I68" t="n">
-        <v>-0.30449915</v>
+        <v>-0.03686841000000002</v>
       </c>
       <c r="J68" t="n">
-        <v>30.449915</v>
+        <v>3.686841000000002</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -6356,13 +6356,13 @@
         <v>0.28</v>
       </c>
       <c r="H69" t="n">
-        <v>0.06899553999999999</v>
+        <v>0.06487846999999999</v>
       </c>
       <c r="I69" t="n">
-        <v>-0.21100446</v>
+        <v>-0.21512153</v>
       </c>
       <c r="J69" t="n">
-        <v>21.100446</v>
+        <v>21.512153</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -6407,13 +6407,13 @@
         <v>0.24</v>
       </c>
       <c r="H70" t="n">
-        <v>0.11074632</v>
+        <v>0.45190441</v>
       </c>
       <c r="I70" t="n">
-        <v>-0.12925368</v>
+        <v>0.21190441</v>
       </c>
       <c r="J70" t="n">
-        <v>12.925368</v>
+        <v>21.190441</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -6458,13 +6458,13 @@
         <v>0.34</v>
       </c>
       <c r="H71" t="n">
-        <v>0.02156874</v>
+        <v>0.05388631</v>
       </c>
       <c r="I71" t="n">
-        <v>-0.31843126</v>
+        <v>-0.28611369</v>
       </c>
       <c r="J71" t="n">
-        <v>31.84312600000001</v>
+        <v>28.611369</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -6509,13 +6509,13 @@
         <v>0.5</v>
       </c>
       <c r="H72" t="n">
-        <v>0.21179647</v>
+        <v>0.11426207</v>
       </c>
       <c r="I72" t="n">
-        <v>-0.28820353</v>
+        <v>-0.38573793</v>
       </c>
       <c r="J72" t="n">
-        <v>28.820353</v>
+        <v>38.573793</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -6560,13 +6560,13 @@
         <v>0.38</v>
       </c>
       <c r="H73" t="n">
-        <v>0.01815125</v>
+        <v>0.10422745</v>
       </c>
       <c r="I73" t="n">
-        <v>-0.36184875</v>
+        <v>-0.27577255</v>
       </c>
       <c r="J73" t="n">
-        <v>36.184875</v>
+        <v>27.577255</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -6611,13 +6611,13 @@
         <v>0.52</v>
       </c>
       <c r="H74" t="n">
-        <v>0.11149217</v>
+        <v>0.15903324</v>
       </c>
       <c r="I74" t="n">
-        <v>-0.40850783</v>
+        <v>-0.3609667600000001</v>
       </c>
       <c r="J74" t="n">
-        <v>40.850783</v>
+        <v>36.096676</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -6662,13 +6662,13 @@
         <v>0.26</v>
       </c>
       <c r="H75" t="n">
-        <v>0.01979482</v>
+        <v>0.0148229</v>
       </c>
       <c r="I75" t="n">
-        <v>-0.24020518</v>
+        <v>-0.2451771</v>
       </c>
       <c r="J75" t="n">
-        <v>24.020518</v>
+        <v>24.51771</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -6713,13 +6713,13 @@
         <v>0.63</v>
       </c>
       <c r="H76" t="n">
-        <v>0.01504631</v>
+        <v>0.11573894</v>
       </c>
       <c r="I76" t="n">
-        <v>-0.61495369</v>
+        <v>-0.51426106</v>
       </c>
       <c r="J76" t="n">
-        <v>61.495369</v>
+        <v>51.426106</v>
       </c>
       <c r="K76" t="inlineStr">
         <is>
@@ -6764,13 +6764,13 @@
         <v>0.5</v>
       </c>
       <c r="H77" t="n">
-        <v>0.00939399</v>
+        <v>0.16870707</v>
       </c>
       <c r="I77" t="n">
-        <v>-0.49060601</v>
+        <v>-0.33129293</v>
       </c>
       <c r="J77" t="n">
-        <v>49.060601</v>
+        <v>33.129293</v>
       </c>
       <c r="K77" t="inlineStr">
         <is>
@@ -6815,13 +6815,13 @@
         <v>0.46</v>
       </c>
       <c r="H78" t="n">
-        <v>0.11601727</v>
+        <v>0.13460228</v>
       </c>
       <c r="I78" t="n">
-        <v>-0.34398273</v>
+        <v>-0.32539772</v>
       </c>
       <c r="J78" t="n">
-        <v>34.398273</v>
+        <v>32.539772</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
@@ -6866,13 +6866,13 @@
         <v>0.28</v>
       </c>
       <c r="H79" t="n">
-        <v>0.13797679</v>
+        <v>0.25992782</v>
       </c>
       <c r="I79" t="n">
-        <v>-0.14202321</v>
+        <v>-0.02007218000000005</v>
       </c>
       <c r="J79" t="n">
-        <v>14.202321</v>
+        <v>2.007218000000005</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
@@ -6917,13 +6917,13 @@
         <v>0.32</v>
       </c>
       <c r="H80" t="n">
-        <v>0.1470067</v>
+        <v>0.48693445</v>
       </c>
       <c r="I80" t="n">
-        <v>-0.1729933</v>
+        <v>0.16693445</v>
       </c>
       <c r="J80" t="n">
-        <v>17.29933</v>
+        <v>16.693445</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
@@ -6968,13 +6968,13 @@
         <v>0.54</v>
       </c>
       <c r="H81" t="n">
-        <v>0.09691590999999999</v>
+        <v>0.19215115</v>
       </c>
       <c r="I81" t="n">
-        <v>-0.44308409</v>
+        <v>-0.34784885</v>
       </c>
       <c r="J81" t="n">
-        <v>44.308409</v>
+        <v>34.784885</v>
       </c>
       <c r="K81" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
casee-v0.4.0-rc3: add probe risk audit
</commit_message>
<xml_diff>
--- a/docs/experiments/casee/results/casee_validation_summary.xlsx
+++ b/docs/experiments/casee/results/casee_validation_summary.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="official_probes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="inlet_profile" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="residuals" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="solid_corner_groups" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2842,7 +2843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M81"/>
+  <dimension ref="A1:O81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2903,10 +2904,20 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>solid_corner_neighbors_max</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>samples</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>solid_corner_risk</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>evidence_type</t>
         </is>
@@ -2954,10 +2965,20 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>3</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3005,10 +3026,20 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3056,10 +3087,20 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3107,10 +3148,20 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3158,10 +3209,20 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3209,10 +3270,20 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3260,10 +3331,20 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3311,10 +3392,20 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3362,10 +3453,20 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3413,10 +3514,20 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3464,10 +3575,20 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3515,10 +3636,20 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3566,10 +3697,20 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3617,10 +3758,20 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3668,10 +3819,20 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3719,10 +3880,20 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3770,10 +3941,20 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3821,10 +4002,20 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3872,10 +4063,20 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3923,10 +4124,20 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -3974,10 +4185,20 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4025,10 +4246,20 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4076,10 +4307,20 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4127,10 +4368,20 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4178,10 +4429,20 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4229,10 +4490,20 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4280,10 +4551,20 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4331,10 +4612,20 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4382,10 +4673,20 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4433,10 +4734,20 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4484,10 +4795,20 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4535,10 +4856,20 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4586,10 +4917,20 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4637,10 +4978,20 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4688,10 +5039,20 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4739,10 +5100,20 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4790,10 +5161,20 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4841,10 +5222,20 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4892,10 +5283,20 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4943,10 +5344,20 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -4994,10 +5405,20 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5045,10 +5466,20 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5096,10 +5527,20 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5147,10 +5588,20 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5198,10 +5649,20 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5249,10 +5710,20 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5300,10 +5771,20 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5351,10 +5832,20 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5402,10 +5893,20 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5453,10 +5954,20 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>3</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5504,10 +6015,20 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5555,10 +6076,20 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5606,10 +6137,20 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5657,10 +6198,20 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5708,10 +6259,20 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5759,10 +6320,20 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5810,10 +6381,20 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5861,10 +6442,20 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5912,10 +6503,20 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -5963,10 +6564,20 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6014,10 +6625,20 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6065,10 +6686,20 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6116,10 +6747,20 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6167,10 +6808,20 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6218,10 +6869,20 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6269,10 +6930,20 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6320,10 +6991,20 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6371,10 +7052,20 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6422,10 +7113,20 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6473,10 +7174,20 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6524,10 +7235,20 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6575,10 +7296,20 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6626,10 +7357,20 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6677,10 +7418,20 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6728,10 +7479,20 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6779,10 +7540,20 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6830,10 +7601,20 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6881,10 +7662,20 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6932,10 +7723,20 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
         <is>
           <t>newly_run</t>
         </is>
@@ -6983,13 +7784,174 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>unknown_until_solver_probe_audit</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
         <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
           <t>newly_run</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>solid_corner_neighbors_max</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>mae_pp</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>rmse_pp</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>bias_pp</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>pearson</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>25</v>
+      </c>
+      <c r="C2" t="n">
+        <v>12.93166104</v>
+      </c>
+      <c r="D2" t="n">
+        <v>15.7918801446684</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-7.094956560000001</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.17647922816893</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.3565835234095897</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>37</v>
+      </c>
+      <c r="C3" t="n">
+        <v>27.11025216216217</v>
+      </c>
+      <c r="D3" t="n">
+        <v>30.98786154726413</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-24.42113054054054</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-3.232167416101973</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-0.1996182930595802</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>13.3376225</v>
+      </c>
+      <c r="D4" t="n">
+        <v>16.97900054858349</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-10.5068685</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-17.0179037267999</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>16</v>
+      </c>
+      <c r="C5" t="n">
+        <v>35.29383725</v>
+      </c>
+      <c r="D5" t="n">
+        <v>39.82934803366287</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-35.29383725</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-3.349962542688314</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.2696392237635756</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
casee-v0.4.0-rc8: add z-center diagnostic
</commit_message>
<xml_diff>
--- a/docs/experiments/casee/results/casee_validation_summary.xlsx
+++ b/docs/experiments/casee/results/casee_validation_summary.xlsx
@@ -2950,13 +2950,13 @@
         <v>0.18</v>
       </c>
       <c r="H2" t="n">
-        <v>0.20830754</v>
+        <v>0.2700105</v>
       </c>
       <c r="I2" t="n">
-        <v>0.02830754000000002</v>
+        <v>0.09001049999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>2.830754000000002</v>
+        <v>9.001049999999999</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -2965,7 +2965,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -3011,13 +3011,13 @@
         <v>0.59</v>
       </c>
       <c r="H3" t="n">
-        <v>0.32874972</v>
+        <v>0.30216974</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.2612502799999999</v>
+        <v>-0.2878302599999999</v>
       </c>
       <c r="J3" t="n">
-        <v>26.12502799999999</v>
+        <v>28.783026</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -3072,13 +3072,13 @@
         <v>0.38</v>
       </c>
       <c r="H4" t="n">
-        <v>0.27719049</v>
+        <v>0.27300675</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.10280951</v>
+        <v>-0.10699325</v>
       </c>
       <c r="J4" t="n">
-        <v>10.280951</v>
+        <v>10.699325</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -3133,13 +3133,13 @@
         <v>0.32</v>
       </c>
       <c r="H5" t="n">
-        <v>0.03532374</v>
+        <v>0.15753856</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.28467626</v>
+        <v>-0.16246144</v>
       </c>
       <c r="J5" t="n">
-        <v>28.467626</v>
+        <v>16.246144</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -3194,13 +3194,13 @@
         <v>0.3</v>
       </c>
       <c r="H6" t="n">
-        <v>0.16671328</v>
+        <v>0.40951982</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.13328672</v>
+        <v>0.10951982</v>
       </c>
       <c r="J6" t="n">
-        <v>13.328672</v>
+        <v>10.951982</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -3209,7 +3209,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -3255,13 +3255,13 @@
         <v>0.34</v>
       </c>
       <c r="H7" t="n">
-        <v>0.11874212</v>
+        <v>0.15472485</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.22125788</v>
+        <v>-0.18527515</v>
       </c>
       <c r="J7" t="n">
-        <v>22.125788</v>
+        <v>18.527515</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -3316,13 +3316,13 @@
         <v>0.26</v>
       </c>
       <c r="H8" t="n">
-        <v>0.25316522</v>
+        <v>0.21382479</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.006834779999999985</v>
+        <v>-0.04617521000000002</v>
       </c>
       <c r="J8" t="n">
-        <v>0.6834779999999985</v>
+        <v>4.617521000000002</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -3341,7 +3341,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -3377,13 +3377,13 @@
         <v>0.14</v>
       </c>
       <c r="H9" t="n">
-        <v>0.04925373</v>
+        <v>0.1812733</v>
       </c>
       <c r="I9" t="n">
-        <v>-0.09074627000000002</v>
+        <v>0.04127329999999998</v>
       </c>
       <c r="J9" t="n">
-        <v>9.074627000000001</v>
+        <v>4.127329999999999</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -3392,7 +3392,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -3438,13 +3438,13 @@
         <v>0.12</v>
       </c>
       <c r="H10" t="n">
-        <v>0.08338690999999999</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.03661309</v>
+        <v>-0.12</v>
       </c>
       <c r="J10" t="n">
-        <v>3.661309</v>
+        <v>12</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -3453,7 +3453,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -3463,7 +3463,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>high</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -3499,13 +3499,13 @@
         <v>0.1</v>
       </c>
       <c r="H11" t="n">
-        <v>0.31200519</v>
+        <v>0.29147353</v>
       </c>
       <c r="I11" t="n">
-        <v>0.21200519</v>
+        <v>0.19147353</v>
       </c>
       <c r="J11" t="n">
-        <v>21.200519</v>
+        <v>19.147353</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -3560,13 +3560,13 @@
         <v>0.55</v>
       </c>
       <c r="H12" t="n">
-        <v>0.22062139</v>
+        <v>0.66346047</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.32937861</v>
+        <v>0.1134604699999999</v>
       </c>
       <c r="J12" t="n">
-        <v>32.937861</v>
+        <v>11.34604699999999</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -3585,7 +3585,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -3621,13 +3621,13 @@
         <v>0.3</v>
       </c>
       <c r="H13" t="n">
-        <v>0.2657773</v>
+        <v>0.30810005</v>
       </c>
       <c r="I13" t="n">
-        <v>-0.03422269999999999</v>
+        <v>0.008100050000000025</v>
       </c>
       <c r="J13" t="n">
-        <v>3.422269999999999</v>
+        <v>0.8100050000000025</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -3682,13 +3682,13 @@
         <v>0.59</v>
       </c>
       <c r="H14" t="n">
-        <v>0.11199946</v>
+        <v>0.26613972</v>
       </c>
       <c r="I14" t="n">
-        <v>-0.47800054</v>
+        <v>-0.3238602799999999</v>
       </c>
       <c r="J14" t="n">
-        <v>47.800054</v>
+        <v>32.386028</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -3697,7 +3697,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -3707,7 +3707,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -3743,13 +3743,13 @@
         <v>0.46</v>
       </c>
       <c r="H15" t="n">
-        <v>0.37454433</v>
+        <v>0.39071817</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.08545567000000004</v>
+        <v>-0.06928183000000004</v>
       </c>
       <c r="J15" t="n">
-        <v>8.545567000000004</v>
+        <v>6.928183000000004</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -3804,13 +3804,13 @@
         <v>0.4</v>
       </c>
       <c r="H16" t="n">
-        <v>0.384069</v>
+        <v>0.32245237</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.01593100000000003</v>
+        <v>-0.07754763000000003</v>
       </c>
       <c r="J16" t="n">
-        <v>1.593100000000003</v>
+        <v>7.754763000000003</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -3865,13 +3865,13 @@
         <v>0.38</v>
       </c>
       <c r="H17" t="n">
-        <v>0.23438932</v>
+        <v>0.13387697</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.14561068</v>
+        <v>-0.24612303</v>
       </c>
       <c r="J17" t="n">
-        <v>14.561068</v>
+        <v>24.612303</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -3926,13 +3926,13 @@
         <v>0.2</v>
       </c>
       <c r="H18" t="n">
-        <v>0.09064137</v>
+        <v>0.41019039</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.10935863</v>
+        <v>0.21019039</v>
       </c>
       <c r="J18" t="n">
-        <v>10.935863</v>
+        <v>21.019039</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -3941,7 +3941,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -3987,13 +3987,13 @@
         <v>0.28</v>
       </c>
       <c r="H19" t="n">
-        <v>0.16247229</v>
+        <v>0.36002944</v>
       </c>
       <c r="I19" t="n">
-        <v>-0.11752771</v>
+        <v>0.08002943999999995</v>
       </c>
       <c r="J19" t="n">
-        <v>11.752771</v>
+        <v>8.002943999999996</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -4002,7 +4002,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -4048,13 +4048,13 @@
         <v>0.32</v>
       </c>
       <c r="H20" t="n">
-        <v>0.03496582</v>
+        <v>0.19919757</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.28503418</v>
+        <v>-0.12080243</v>
       </c>
       <c r="J20" t="n">
-        <v>28.503418</v>
+        <v>12.080243</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -4109,13 +4109,13 @@
         <v>0.2</v>
       </c>
       <c r="H21" t="n">
-        <v>0.18146655</v>
+        <v>0.32006538</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.01853345000000001</v>
+        <v>0.12006538</v>
       </c>
       <c r="J21" t="n">
-        <v>1.853345000000001</v>
+        <v>12.006538</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -4124,7 +4124,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -4134,7 +4134,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -4170,13 +4170,13 @@
         <v>0.4</v>
       </c>
       <c r="H22" t="n">
-        <v>0.2651739</v>
+        <v>0.32024781</v>
       </c>
       <c r="I22" t="n">
-        <v>-0.1348261</v>
+        <v>-0.07975219</v>
       </c>
       <c r="J22" t="n">
-        <v>13.48261</v>
+        <v>7.975219</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -4231,13 +4231,13 @@
         <v>0.59</v>
       </c>
       <c r="H23" t="n">
-        <v>0.16242976</v>
+        <v>0.16300356</v>
       </c>
       <c r="I23" t="n">
-        <v>-0.42757024</v>
+        <v>-0.42699644</v>
       </c>
       <c r="J23" t="n">
-        <v>42.757024</v>
+        <v>42.699644</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -4292,13 +4292,13 @@
         <v>0.54</v>
       </c>
       <c r="H24" t="n">
-        <v>0.15774745</v>
+        <v>0.12600656</v>
       </c>
       <c r="I24" t="n">
-        <v>-0.38225255</v>
+        <v>-0.41399344</v>
       </c>
       <c r="J24" t="n">
-        <v>38.225255</v>
+        <v>41.39934400000001</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -4353,13 +4353,13 @@
         <v>0.46</v>
       </c>
       <c r="H25" t="n">
-        <v>0.19116407</v>
+        <v>0.28048573</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.2688359300000001</v>
+        <v>-0.17951427</v>
       </c>
       <c r="J25" t="n">
-        <v>26.883593</v>
+        <v>17.951427</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -4414,13 +4414,13 @@
         <v>0.52</v>
       </c>
       <c r="H26" t="n">
-        <v>0.38581118</v>
+        <v>0.36917086</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.13418882</v>
+        <v>-0.15082914</v>
       </c>
       <c r="J26" t="n">
-        <v>13.418882</v>
+        <v>15.082914</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -4475,13 +4475,13 @@
         <v>0.55</v>
       </c>
       <c r="H27" t="n">
-        <v>0.35554295</v>
+        <v>0.45826083</v>
       </c>
       <c r="I27" t="n">
-        <v>-0.19445705</v>
+        <v>-0.09173917000000004</v>
       </c>
       <c r="J27" t="n">
-        <v>19.445705</v>
+        <v>9.173917000000003</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -4536,13 +4536,13 @@
         <v>0.48</v>
       </c>
       <c r="H28" t="n">
-        <v>0.19027389</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>-0.28972611</v>
+        <v>-0.48</v>
       </c>
       <c r="J28" t="n">
-        <v>28.972611</v>
+        <v>48</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -4561,7 +4561,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>high</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -4597,13 +4597,13 @@
         <v>0.71</v>
       </c>
       <c r="H29" t="n">
-        <v>0.39362757</v>
+        <v>0.18090167</v>
       </c>
       <c r="I29" t="n">
-        <v>-0.31637243</v>
+        <v>-0.52909833</v>
       </c>
       <c r="J29" t="n">
-        <v>31.637243</v>
+        <v>52.90983299999999</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -4622,7 +4622,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -4658,13 +4658,13 @@
         <v>0.61</v>
       </c>
       <c r="H30" t="n">
-        <v>0.54752525</v>
+        <v>0.01329987</v>
       </c>
       <c r="I30" t="n">
-        <v>-0.06247475000000002</v>
+        <v>-0.59670013</v>
       </c>
       <c r="J30" t="n">
-        <v>6.247475000000002</v>
+        <v>59.670013</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -4719,13 +4719,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="H31" t="n">
-        <v>0.18938433</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>-0.50061567</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="J31" t="n">
-        <v>50.061567</v>
+        <v>69</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -4744,7 +4744,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>high</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -4780,13 +4780,13 @@
         <v>0.44</v>
       </c>
       <c r="H32" t="n">
-        <v>0.09889763999999999</v>
+        <v>0.20273667</v>
       </c>
       <c r="I32" t="n">
-        <v>-0.34110236</v>
+        <v>-0.23726333</v>
       </c>
       <c r="J32" t="n">
-        <v>34.110236</v>
+        <v>23.726333</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -4795,7 +4795,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -4805,7 +4805,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -4841,13 +4841,13 @@
         <v>0.54</v>
       </c>
       <c r="H33" t="n">
-        <v>0.20961041</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>-0.33038959</v>
+        <v>-0.54</v>
       </c>
       <c r="J33" t="n">
-        <v>33.038959</v>
+        <v>54</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -4856,7 +4856,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -4866,7 +4866,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>high</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -4902,13 +4902,13 @@
         <v>0.52</v>
       </c>
       <c r="H34" t="n">
-        <v>0.52939261</v>
+        <v>0.542814</v>
       </c>
       <c r="I34" t="n">
-        <v>0.009392610000000023</v>
+        <v>0.022814</v>
       </c>
       <c r="J34" t="n">
-        <v>0.9392610000000023</v>
+        <v>2.2814</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -4963,13 +4963,13 @@
         <v>0.32</v>
       </c>
       <c r="H35" t="n">
-        <v>0.43110631</v>
+        <v>0.35018705</v>
       </c>
       <c r="I35" t="n">
-        <v>0.11110631</v>
+        <v>0.03018704999999999</v>
       </c>
       <c r="J35" t="n">
-        <v>11.110631</v>
+        <v>3.018704999999999</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
@@ -5024,13 +5024,13 @@
         <v>0.5</v>
       </c>
       <c r="H36" t="n">
-        <v>0.39907543</v>
+        <v>0.35114802</v>
       </c>
       <c r="I36" t="n">
-        <v>-0.10092457</v>
+        <v>-0.14885198</v>
       </c>
       <c r="J36" t="n">
-        <v>10.092457</v>
+        <v>14.885198</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -5085,13 +5085,13 @@
         <v>0.32</v>
       </c>
       <c r="H37" t="n">
-        <v>0.42693671</v>
+        <v>0.40088243</v>
       </c>
       <c r="I37" t="n">
-        <v>0.10693671</v>
+        <v>0.08088243000000001</v>
       </c>
       <c r="J37" t="n">
-        <v>10.693671</v>
+        <v>8.088243</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -5146,13 +5146,13 @@
         <v>0.48</v>
       </c>
       <c r="H38" t="n">
-        <v>0.31255821</v>
+        <v>0.28198408</v>
       </c>
       <c r="I38" t="n">
-        <v>-0.16744179</v>
+        <v>-0.19801592</v>
       </c>
       <c r="J38" t="n">
-        <v>16.744179</v>
+        <v>19.801592</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -5207,13 +5207,13 @@
         <v>0.61</v>
       </c>
       <c r="H39" t="n">
-        <v>0.11995387</v>
+        <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>-0.49004613</v>
+        <v>-0.61</v>
       </c>
       <c r="J39" t="n">
-        <v>49.004613</v>
+        <v>61</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -5222,7 +5222,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>high</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -5268,13 +5268,13 @@
         <v>0.26</v>
       </c>
       <c r="H40" t="n">
-        <v>0.36592446</v>
+        <v>0.41252098</v>
       </c>
       <c r="I40" t="n">
-        <v>0.10592446</v>
+        <v>0.15252098</v>
       </c>
       <c r="J40" t="n">
-        <v>10.592446</v>
+        <v>15.252098</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -5283,7 +5283,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -5293,7 +5293,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
@@ -5329,13 +5329,13 @@
         <v>0.38</v>
       </c>
       <c r="H41" t="n">
-        <v>0.07938853</v>
+        <v>0.39988811</v>
       </c>
       <c r="I41" t="n">
-        <v>-0.30061147</v>
+        <v>0.01988811000000001</v>
       </c>
       <c r="J41" t="n">
-        <v>30.061147</v>
+        <v>1.988811000000001</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -5344,7 +5344,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -5354,7 +5354,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
@@ -5390,13 +5390,13 @@
         <v>0.46</v>
       </c>
       <c r="H42" t="n">
-        <v>0.10755455</v>
+        <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>-0.35244545</v>
+        <v>-0.46</v>
       </c>
       <c r="J42" t="n">
-        <v>35.244545</v>
+        <v>46</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -5451,13 +5451,13 @@
         <v>0.44</v>
       </c>
       <c r="H43" t="n">
-        <v>0.11130642</v>
+        <v>0.34939494</v>
       </c>
       <c r="I43" t="n">
-        <v>-0.32869358</v>
+        <v>-0.09060506000000002</v>
       </c>
       <c r="J43" t="n">
-        <v>32.869358</v>
+        <v>9.060506000000002</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -5466,7 +5466,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -5476,7 +5476,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
@@ -5512,13 +5512,13 @@
         <v>0.3</v>
       </c>
       <c r="H44" t="n">
-        <v>0.1573176</v>
+        <v>0.31412336</v>
       </c>
       <c r="I44" t="n">
-        <v>-0.1426824</v>
+        <v>0.01412336000000003</v>
       </c>
       <c r="J44" t="n">
-        <v>14.26824</v>
+        <v>1.412336000000003</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -5527,7 +5527,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -5537,7 +5537,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -5573,13 +5573,13 @@
         <v>0.46</v>
       </c>
       <c r="H45" t="n">
-        <v>0.21231887</v>
+        <v>0.61101136</v>
       </c>
       <c r="I45" t="n">
-        <v>-0.24768113</v>
+        <v>0.15101136</v>
       </c>
       <c r="J45" t="n">
-        <v>24.768113</v>
+        <v>15.101136</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -5588,7 +5588,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -5598,7 +5598,7 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
@@ -5634,13 +5634,13 @@
         <v>0.2</v>
       </c>
       <c r="H46" t="n">
-        <v>0.27860525</v>
+        <v>0.23534922</v>
       </c>
       <c r="I46" t="n">
-        <v>0.07860525000000002</v>
+        <v>0.03534921999999999</v>
       </c>
       <c r="J46" t="n">
-        <v>7.860525000000002</v>
+        <v>3.534921999999999</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
@@ -5695,13 +5695,13 @@
         <v>0.18</v>
       </c>
       <c r="H47" t="n">
-        <v>0.35965863</v>
+        <v>0.00581474</v>
       </c>
       <c r="I47" t="n">
-        <v>0.17965863</v>
+        <v>-0.17418526</v>
       </c>
       <c r="J47" t="n">
-        <v>17.965863</v>
+        <v>17.418526</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
@@ -5710,7 +5710,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -5720,7 +5720,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>high</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
@@ -5756,13 +5756,13 @@
         <v>0.2</v>
       </c>
       <c r="H48" t="n">
-        <v>0.00147794</v>
+        <v>0.00040261</v>
       </c>
       <c r="I48" t="n">
-        <v>-0.19852206</v>
+        <v>-0.19959739</v>
       </c>
       <c r="J48" t="n">
-        <v>19.852206</v>
+        <v>19.959739</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -5817,13 +5817,13 @@
         <v>0.36</v>
       </c>
       <c r="H49" t="n">
-        <v>0.336626</v>
+        <v>0</v>
       </c>
       <c r="I49" t="n">
-        <v>-0.02337400000000001</v>
+        <v>-0.36</v>
       </c>
       <c r="J49" t="n">
-        <v>2.337400000000001</v>
+        <v>36</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
@@ -5878,13 +5878,13 @@
         <v>0.3</v>
       </c>
       <c r="H50" t="n">
-        <v>0.26429585</v>
+        <v>0.089948</v>
       </c>
       <c r="I50" t="n">
-        <v>-0.03570414999999999</v>
+        <v>-0.210052</v>
       </c>
       <c r="J50" t="n">
-        <v>3.570414999999999</v>
+        <v>21.0052</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
@@ -5893,7 +5893,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>high</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
@@ -5939,13 +5939,13 @@
         <v>0.26</v>
       </c>
       <c r="H51" t="n">
-        <v>0.02155509</v>
+        <v>0.08481619999999999</v>
       </c>
       <c r="I51" t="n">
-        <v>-0.23844491</v>
+        <v>-0.1751838</v>
       </c>
       <c r="J51" t="n">
-        <v>23.844491</v>
+        <v>17.51838</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -5954,7 +5954,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -6000,13 +6000,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="H52" t="n">
-        <v>0.26060797</v>
+        <v>0.48384602</v>
       </c>
       <c r="I52" t="n">
-        <v>-0.4293920299999999</v>
+        <v>-0.20615398</v>
       </c>
       <c r="J52" t="n">
-        <v>42.93920299999999</v>
+        <v>20.615398</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -6025,7 +6025,7 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
@@ -6061,13 +6061,13 @@
         <v>0.63</v>
       </c>
       <c r="H53" t="n">
-        <v>0.09783202000000001</v>
+        <v>0.29702716</v>
       </c>
       <c r="I53" t="n">
-        <v>-0.53216798</v>
+        <v>-0.33297284</v>
       </c>
       <c r="J53" t="n">
-        <v>53.216798</v>
+        <v>33.297284</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -6076,7 +6076,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -6122,13 +6122,13 @@
         <v>0.57</v>
       </c>
       <c r="H54" t="n">
-        <v>0.16324099</v>
+        <v>0.29621709</v>
       </c>
       <c r="I54" t="n">
-        <v>-0.4067590099999999</v>
+        <v>-0.2737829099999999</v>
       </c>
       <c r="J54" t="n">
-        <v>40.67590099999999</v>
+        <v>27.37829099999999</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -6137,7 +6137,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -6147,7 +6147,7 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
@@ -6183,13 +6183,13 @@
         <v>0.59</v>
       </c>
       <c r="H55" t="n">
-        <v>0.04225041</v>
+        <v>0.55412208</v>
       </c>
       <c r="I55" t="n">
-        <v>-0.54774959</v>
+        <v>-0.03587792000000001</v>
       </c>
       <c r="J55" t="n">
-        <v>54.774959</v>
+        <v>3.587792000000001</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -6208,7 +6208,7 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
@@ -6244,13 +6244,13 @@
         <v>0.38</v>
       </c>
       <c r="H56" t="n">
-        <v>0.29619185</v>
+        <v>0.42488302</v>
       </c>
       <c r="I56" t="n">
-        <v>-0.08380815000000003</v>
+        <v>0.04488302</v>
       </c>
       <c r="J56" t="n">
-        <v>8.380815000000002</v>
+        <v>4.488301999999999</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
@@ -6259,7 +6259,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -6269,7 +6269,7 @@
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
@@ -6305,13 +6305,13 @@
         <v>0.67</v>
       </c>
       <c r="H57" t="n">
-        <v>0.20379514</v>
+        <v>0.23035676</v>
       </c>
       <c r="I57" t="n">
-        <v>-0.4662048600000001</v>
+        <v>-0.43964324</v>
       </c>
       <c r="J57" t="n">
-        <v>46.62048600000001</v>
+        <v>43.964324</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
@@ -6366,13 +6366,13 @@
         <v>0.34</v>
       </c>
       <c r="H58" t="n">
-        <v>0.38460754</v>
+        <v>0.38878271</v>
       </c>
       <c r="I58" t="n">
-        <v>0.04460754</v>
+        <v>0.04878270999999995</v>
       </c>
       <c r="J58" t="n">
-        <v>4.460754</v>
+        <v>4.878270999999995</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -6427,13 +6427,13 @@
         <v>0.85</v>
       </c>
       <c r="H59" t="n">
-        <v>0.10843476</v>
+        <v>0.03546029</v>
       </c>
       <c r="I59" t="n">
-        <v>-0.74156524</v>
+        <v>-0.81453971</v>
       </c>
       <c r="J59" t="n">
-        <v>74.156524</v>
+        <v>81.453971</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
@@ -6442,7 +6442,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -6452,7 +6452,7 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
@@ -6488,13 +6488,13 @@
         <v>0.42</v>
       </c>
       <c r="H60" t="n">
-        <v>0.13367753</v>
+        <v>0.3738214</v>
       </c>
       <c r="I60" t="n">
-        <v>-0.28632247</v>
+        <v>-0.04617859999999996</v>
       </c>
       <c r="J60" t="n">
-        <v>28.632247</v>
+        <v>4.617859999999996</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
@@ -6503,7 +6503,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -6513,7 +6513,7 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
@@ -6549,13 +6549,13 @@
         <v>0.73</v>
       </c>
       <c r="H61" t="n">
-        <v>0.39983383</v>
+        <v>0.40659553</v>
       </c>
       <c r="I61" t="n">
-        <v>-0.33016617</v>
+        <v>-0.32340447</v>
       </c>
       <c r="J61" t="n">
-        <v>33.016617</v>
+        <v>32.340447</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
@@ -6610,13 +6610,13 @@
         <v>0.54</v>
       </c>
       <c r="H62" t="n">
-        <v>0.01660191</v>
+        <v>0</v>
       </c>
       <c r="I62" t="n">
-        <v>-0.52339809</v>
+        <v>-0.54</v>
       </c>
       <c r="J62" t="n">
-        <v>52.339809</v>
+        <v>54</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -6671,13 +6671,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="H63" t="n">
-        <v>0.02344557</v>
+        <v>0.13480377</v>
       </c>
       <c r="I63" t="n">
-        <v>-0.6665544299999999</v>
+        <v>-0.55519623</v>
       </c>
       <c r="J63" t="n">
-        <v>66.65544299999999</v>
+        <v>55.519623</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -6696,7 +6696,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
@@ -6732,13 +6732,13 @@
         <v>0.4</v>
       </c>
       <c r="H64" t="n">
-        <v>0.25829743</v>
+        <v>0.50945962</v>
       </c>
       <c r="I64" t="n">
-        <v>-0.14170257</v>
+        <v>0.10945962</v>
       </c>
       <c r="J64" t="n">
-        <v>14.170257</v>
+        <v>10.945962</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
@@ -6747,7 +6747,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -6757,7 +6757,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
@@ -6793,13 +6793,13 @@
         <v>0.44</v>
       </c>
       <c r="H65" t="n">
-        <v>0.33534344</v>
+        <v>0.32212837</v>
       </c>
       <c r="I65" t="n">
-        <v>-0.10465656</v>
+        <v>-0.11787163</v>
       </c>
       <c r="J65" t="n">
-        <v>10.465656</v>
+        <v>11.787163</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -6854,13 +6854,13 @@
         <v>0.3</v>
       </c>
       <c r="H66" t="n">
-        <v>0.05556118</v>
+        <v>0</v>
       </c>
       <c r="I66" t="n">
-        <v>-0.24443882</v>
+        <v>-0.3</v>
       </c>
       <c r="J66" t="n">
-        <v>24.443882</v>
+        <v>30</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
@@ -6915,13 +6915,13 @@
         <v>0.32</v>
       </c>
       <c r="H67" t="n">
-        <v>0.01333601</v>
+        <v>0.41141345</v>
       </c>
       <c r="I67" t="n">
-        <v>-0.30666399</v>
+        <v>0.09141345000000001</v>
       </c>
       <c r="J67" t="n">
-        <v>30.666399</v>
+        <v>9.141345000000001</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -6930,7 +6930,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -6940,7 +6940,7 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
@@ -6976,13 +6976,13 @@
         <v>0.5</v>
       </c>
       <c r="H68" t="n">
-        <v>0.46313159</v>
+        <v>0</v>
       </c>
       <c r="I68" t="n">
-        <v>-0.03686841000000002</v>
+        <v>-0.5</v>
       </c>
       <c r="J68" t="n">
-        <v>3.686841000000002</v>
+        <v>50</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -6991,7 +6991,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -7001,7 +7001,7 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>high</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
@@ -7037,13 +7037,13 @@
         <v>0.28</v>
       </c>
       <c r="H69" t="n">
-        <v>0.06487846999999999</v>
+        <v>0.07076399</v>
       </c>
       <c r="I69" t="n">
-        <v>-0.21512153</v>
+        <v>-0.20923601</v>
       </c>
       <c r="J69" t="n">
-        <v>21.512153</v>
+        <v>20.923601</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -7052,7 +7052,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -7062,7 +7062,7 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -7098,13 +7098,13 @@
         <v>0.24</v>
       </c>
       <c r="H70" t="n">
-        <v>0.45190441</v>
+        <v>0</v>
       </c>
       <c r="I70" t="n">
-        <v>0.21190441</v>
+        <v>-0.24</v>
       </c>
       <c r="J70" t="n">
-        <v>21.190441</v>
+        <v>24</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -7159,13 +7159,13 @@
         <v>0.34</v>
       </c>
       <c r="H71" t="n">
-        <v>0.05388631</v>
+        <v>0.40547651</v>
       </c>
       <c r="I71" t="n">
-        <v>-0.28611369</v>
+        <v>0.06547650999999999</v>
       </c>
       <c r="J71" t="n">
-        <v>28.611369</v>
+        <v>6.547650999999998</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -7174,7 +7174,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
@@ -7220,13 +7220,13 @@
         <v>0.5</v>
       </c>
       <c r="H72" t="n">
-        <v>0.11426207</v>
+        <v>0.21498994</v>
       </c>
       <c r="I72" t="n">
-        <v>-0.38573793</v>
+        <v>-0.28501006</v>
       </c>
       <c r="J72" t="n">
-        <v>38.573793</v>
+        <v>28.501006</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -7235,7 +7235,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -7245,7 +7245,7 @@
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
@@ -7281,13 +7281,13 @@
         <v>0.38</v>
       </c>
       <c r="H73" t="n">
-        <v>0.10422745</v>
+        <v>0.21286575</v>
       </c>
       <c r="I73" t="n">
-        <v>-0.27577255</v>
+        <v>-0.16713425</v>
       </c>
       <c r="J73" t="n">
-        <v>27.577255</v>
+        <v>16.713425</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -7296,7 +7296,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -7306,7 +7306,7 @@
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
@@ -7342,13 +7342,13 @@
         <v>0.52</v>
       </c>
       <c r="H74" t="n">
-        <v>0.15903324</v>
+        <v>0.36781015</v>
       </c>
       <c r="I74" t="n">
-        <v>-0.3609667600000001</v>
+        <v>-0.15218985</v>
       </c>
       <c r="J74" t="n">
-        <v>36.096676</v>
+        <v>15.218985</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -7357,7 +7357,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -7367,7 +7367,7 @@
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
@@ -7403,13 +7403,13 @@
         <v>0.26</v>
       </c>
       <c r="H75" t="n">
-        <v>0.0148229</v>
+        <v>0.07734399</v>
       </c>
       <c r="I75" t="n">
-        <v>-0.2451771</v>
+        <v>-0.18265601</v>
       </c>
       <c r="J75" t="n">
-        <v>24.51771</v>
+        <v>18.265601</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -7464,13 +7464,13 @@
         <v>0.63</v>
       </c>
       <c r="H76" t="n">
-        <v>0.11573894</v>
+        <v>0.59151069</v>
       </c>
       <c r="I76" t="n">
-        <v>-0.51426106</v>
+        <v>-0.03848931</v>
       </c>
       <c r="J76" t="n">
-        <v>51.426106</v>
+        <v>3.848931</v>
       </c>
       <c r="K76" t="inlineStr">
         <is>
@@ -7479,7 +7479,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -7489,7 +7489,7 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
@@ -7525,13 +7525,13 @@
         <v>0.5</v>
       </c>
       <c r="H77" t="n">
-        <v>0.16870707</v>
+        <v>0.54996215</v>
       </c>
       <c r="I77" t="n">
-        <v>-0.33129293</v>
+        <v>0.04996215000000004</v>
       </c>
       <c r="J77" t="n">
-        <v>33.129293</v>
+        <v>4.996215000000004</v>
       </c>
       <c r="K77" t="inlineStr">
         <is>
@@ -7540,7 +7540,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -7550,7 +7550,7 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
@@ -7586,13 +7586,13 @@
         <v>0.46</v>
       </c>
       <c r="H78" t="n">
-        <v>0.13460228</v>
+        <v>0.41840826</v>
       </c>
       <c r="I78" t="n">
-        <v>-0.32539772</v>
+        <v>-0.04159174000000004</v>
       </c>
       <c r="J78" t="n">
-        <v>32.539772</v>
+        <v>4.159174000000005</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
@@ -7601,7 +7601,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
@@ -7647,13 +7647,13 @@
         <v>0.28</v>
       </c>
       <c r="H79" t="n">
-        <v>0.25992782</v>
+        <v>0.26845467</v>
       </c>
       <c r="I79" t="n">
-        <v>-0.02007218000000005</v>
+        <v>-0.01154533000000002</v>
       </c>
       <c r="J79" t="n">
-        <v>2.007218000000005</v>
+        <v>1.154533000000002</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
@@ -7662,7 +7662,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -7672,7 +7672,7 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
@@ -7708,13 +7708,13 @@
         <v>0.32</v>
       </c>
       <c r="H80" t="n">
-        <v>0.48693445</v>
+        <v>0.01693663</v>
       </c>
       <c r="I80" t="n">
-        <v>0.16693445</v>
+        <v>-0.30306337</v>
       </c>
       <c r="J80" t="n">
-        <v>16.693445</v>
+        <v>30.306337</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>moderate</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
@@ -7769,13 +7769,13 @@
         <v>0.54</v>
       </c>
       <c r="H81" t="n">
-        <v>0.19215115</v>
+        <v>0.43701617</v>
       </c>
       <c r="I81" t="n">
-        <v>-0.34784885</v>
+        <v>-0.1029838300000001</v>
       </c>
       <c r="J81" t="n">
-        <v>34.784885</v>
+        <v>10.298383</v>
       </c>
       <c r="K81" t="inlineStr">
         <is>
@@ -7784,7 +7784,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
@@ -7794,7 +7794,7 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>moderate</t>
+          <t>none</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
@@ -7814,7 +7814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7861,22 +7861,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="C2" t="n">
-        <v>12.93166104</v>
+        <v>12.43470282978723</v>
       </c>
       <c r="D2" t="n">
-        <v>15.7918801446684</v>
+        <v>15.38198413511713</v>
       </c>
       <c r="E2" t="n">
-        <v>-7.094956560000001</v>
+        <v>-5.378619425531916</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.17647922816893</v>
+        <v>-0.2810391422898797</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3565835234095897</v>
+        <v>0.3225991736103837</v>
       </c>
     </row>
     <row r="3">
@@ -7886,72 +7886,47 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="C3" t="n">
-        <v>27.11025216216217</v>
+        <v>31.92497645</v>
       </c>
       <c r="D3" t="n">
-        <v>30.98786154726413</v>
+        <v>37.81412006355944</v>
       </c>
       <c r="E3" t="n">
-        <v>-24.42113054054054</v>
+        <v>-29.69800395</v>
       </c>
       <c r="F3" t="n">
-        <v>-3.232167416101973</v>
+        <v>-2.746253965734728</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1996182930595802</v>
+        <v>-0.1355037016694693</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C4" t="n">
-        <v>13.3376225</v>
+        <v>35.844776</v>
       </c>
       <c r="D4" t="n">
-        <v>16.97900054858349</v>
+        <v>40.91063484527469</v>
       </c>
       <c r="E4" t="n">
-        <v>-10.5068685</v>
+        <v>-35.844776</v>
       </c>
       <c r="F4" t="n">
-        <v>-17.0179037267999</v>
+        <v>-4.513467844176351</v>
       </c>
       <c r="G4" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>16</v>
-      </c>
-      <c r="C5" t="n">
-        <v>35.29383725</v>
-      </c>
-      <c r="D5" t="n">
-        <v>39.82934803366287</v>
-      </c>
-      <c r="E5" t="n">
-        <v>-35.29383725</v>
-      </c>
-      <c r="F5" t="n">
-        <v>-3.349962542688314</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.2696392237635756</v>
+        <v>-0.2544653157700059</v>
       </c>
     </row>
   </sheetData>

</xml_diff>